<commit_message>
add a alpha delta figures under different parameters
</commit_message>
<xml_diff>
--- a/KLexperiments_ME_FLP_PD.xlsx
+++ b/KLexperiments_ME_FLP_PD.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ME3CodeAI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20EF5BFF-C4A4-434B-B881-D58320D5B6F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15F3AE2C-DFE0-4CF1-BDB3-E5FAD48E3B1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="171">
   <si>
     <t>run_number</t>
   </si>
@@ -553,6 +553,12 @@
   </si>
   <si>
     <t>P25</t>
+  </si>
+  <si>
+    <t>a variant of P17 with lower kappa</t>
+  </si>
+  <si>
+    <t>P26</t>
   </si>
 </sst>
 </file>
@@ -1128,7 +1134,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O72"/>
+  <dimension ref="A1:O73"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.453125" customWidth="1"/>
@@ -4429,73 +4435,120 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A71">
+    <row r="71" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A71" s="31">
+        <v>70</v>
+      </c>
+      <c r="B71" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="C71" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="D71" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="E71" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="F71">
+        <v>26</v>
+      </c>
+      <c r="G71" s="21">
+        <v>5</v>
+      </c>
+      <c r="H71" s="21">
+        <v>4</v>
+      </c>
+      <c r="I71" s="19">
+        <v>1</v>
+      </c>
+      <c r="J71" s="19">
+        <v>1</v>
+      </c>
+      <c r="K71" s="19">
+        <v>2</v>
+      </c>
+      <c r="L71" s="21">
+        <v>13</v>
+      </c>
+      <c r="M71" s="19">
+        <v>2</v>
+      </c>
+      <c r="N71" s="19">
+        <v>1</v>
+      </c>
+      <c r="O71" s="19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A72">
         <v>10000</v>
       </c>
-      <c r="E71" t="s">
+      <c r="E72" t="s">
         <v>23</v>
       </c>
-      <c r="F71" t="s">
+      <c r="F72" t="s">
         <v>24</v>
       </c>
-      <c r="G71" t="s">
+      <c r="G72" t="s">
         <v>25</v>
       </c>
-      <c r="H71" t="s">
+      <c r="H72" t="s">
         <v>26</v>
       </c>
-      <c r="I71" t="s">
+      <c r="I72" t="s">
         <v>27</v>
       </c>
-      <c r="J71" t="s">
+      <c r="J72" t="s">
         <v>28</v>
       </c>
-      <c r="K71" t="s">
+      <c r="K72" t="s">
         <v>29</v>
       </c>
-      <c r="L71" t="s">
+      <c r="L72" t="s">
         <v>30</v>
       </c>
-      <c r="M71" t="s">
+      <c r="M72" t="s">
         <v>31</v>
       </c>
-      <c r="N71" t="s">
+      <c r="N72" t="s">
         <v>32</v>
       </c>
-      <c r="O71" t="s">
+      <c r="O72" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="F72">
-        <v>1</v>
-      </c>
-      <c r="G72">
-        <v>2</v>
-      </c>
-      <c r="H72">
+    <row r="73" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="F73">
+        <v>1</v>
+      </c>
+      <c r="G73">
+        <v>2</v>
+      </c>
+      <c r="H73">
         <v>3</v>
       </c>
-      <c r="I72">
+      <c r="I73">
         <v>4</v>
       </c>
-      <c r="J72">
+      <c r="J73">
         <v>5</v>
       </c>
-      <c r="K72">
+      <c r="K73">
         <v>6</v>
       </c>
-      <c r="L72">
+      <c r="L73">
         <v>7</v>
       </c>
-      <c r="M72">
+      <c r="M73">
         <v>8</v>
       </c>
-      <c r="N72">
+      <c r="N73">
         <v>9</v>
       </c>
-      <c r="O72">
+      <c r="O73">
         <v>10</v>
       </c>
     </row>
@@ -4550,7 +4603,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:P26"/>
+  <dimension ref="A1:P27"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.7265625" customWidth="1"/>
@@ -5567,7 +5620,7 @@
         <v>0.08</v>
       </c>
       <c r="P20">
-        <f>1.5/400</f>
+        <f t="shared" ref="P20:P26" si="0">1.5/400</f>
         <v>3.7499999999999999E-3</v>
       </c>
     </row>
@@ -5618,7 +5671,7 @@
         <v>0.08</v>
       </c>
       <c r="P21">
-        <f>1.5/400</f>
+        <f t="shared" si="0"/>
         <v>3.7499999999999999E-3</v>
       </c>
     </row>
@@ -5669,7 +5722,7 @@
         <v>0.08</v>
       </c>
       <c r="P22">
-        <f>1.5/400</f>
+        <f t="shared" si="0"/>
         <v>3.7499999999999999E-3</v>
       </c>
     </row>
@@ -5720,7 +5773,7 @@
         <v>0.08</v>
       </c>
       <c r="P23">
-        <f>1.5/400</f>
+        <f t="shared" si="0"/>
         <v>3.7499999999999999E-3</v>
       </c>
     </row>
@@ -5771,7 +5824,7 @@
         <v>0.08</v>
       </c>
       <c r="P24">
-        <f>1.5/400</f>
+        <f t="shared" si="0"/>
         <v>3.7499999999999999E-3</v>
       </c>
     </row>
@@ -5822,7 +5875,7 @@
         <v>0.08</v>
       </c>
       <c r="P25">
-        <f>1.5/400</f>
+        <f t="shared" si="0"/>
         <v>3.7499999999999999E-3</v>
       </c>
     </row>
@@ -5873,6 +5926,57 @@
         <v>0.08</v>
       </c>
       <c r="P26">
+        <f t="shared" si="0"/>
+        <v>3.7499999999999999E-3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>170</v>
+      </c>
+      <c r="B27" t="s">
+        <v>169</v>
+      </c>
+      <c r="C27">
+        <v>1</v>
+      </c>
+      <c r="D27" s="28">
+        <v>0.1</v>
+      </c>
+      <c r="E27">
+        <v>0</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+      <c r="G27">
+        <v>1.7299999999999999E-2</v>
+      </c>
+      <c r="H27">
+        <v>1</v>
+      </c>
+      <c r="I27" s="27">
+        <v>0.1</v>
+      </c>
+      <c r="J27">
+        <v>0</v>
+      </c>
+      <c r="K27">
+        <v>0</v>
+      </c>
+      <c r="L27">
+        <v>1.7299999999999999E-2</v>
+      </c>
+      <c r="M27">
+        <v>0.995</v>
+      </c>
+      <c r="N27">
+        <v>0.995</v>
+      </c>
+      <c r="O27">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="P27">
         <f>1.5/400</f>
         <v>3.7499999999999999E-3</v>
       </c>

</xml_diff>

<commit_message>
added plots from experiment 71 72 73
</commit_message>
<xml_diff>
--- a/KLexperiments_ME_FLP_PD.xlsx
+++ b/KLexperiments_ME_FLP_PD.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ME3CodeAI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ME3codeAI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15F3AE2C-DFE0-4CF1-BDB3-E5FAD48E3B1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7B52F4F-D1BF-418F-9291-7BA7D0E6B008}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RUN_info" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="175">
   <si>
     <t>run_number</t>
   </si>
@@ -559,6 +559,18 @@
   </si>
   <si>
     <t>P26</t>
+  </si>
+  <si>
+    <t>P27</t>
+  </si>
+  <si>
+    <t>a variant of P17 with even higher vtheta_x1</t>
+  </si>
+  <si>
+    <t>S8</t>
+  </si>
+  <si>
+    <t>S9</t>
   </si>
 </sst>
 </file>
@@ -1134,18 +1146,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O73"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:O76"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.453125" customWidth="1"/>
-    <col min="2" max="3" width="8.7265625" customWidth="1"/>
-    <col min="4" max="4" width="11.26953125" customWidth="1"/>
-    <col min="5" max="5" width="8.7265625" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" customWidth="1"/>
+    <col min="2" max="3" width="8.7109375" customWidth="1"/>
+    <col min="4" max="4" width="11.28515625" customWidth="1"/>
+    <col min="5" max="5" width="8.7109375" customWidth="1"/>
     <col min="6" max="10" width="12" customWidth="1"/>
-    <col min="11" max="1025" width="8.7265625" customWidth="1"/>
+    <col min="11" max="1025" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1192,7 +1204,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1239,7 +1251,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1286,7 +1298,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1333,7 +1345,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1380,7 +1392,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1427,7 +1439,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1474,7 +1486,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1521,7 +1533,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1568,7 +1580,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1615,7 +1627,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1662,7 +1674,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1709,7 +1721,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1756,7 +1768,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -1803,7 +1815,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -1850,7 +1862,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1897,7 +1909,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4">
         <v>16</v>
       </c>
@@ -1944,7 +1956,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4">
         <v>17</v>
       </c>
@@ -1991,7 +2003,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -2038,7 +2050,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="6">
         <v>19</v>
       </c>
@@ -2085,7 +2097,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -2132,7 +2144,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="6">
         <v>21</v>
       </c>
@@ -2179,7 +2191,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="8">
         <v>22</v>
       </c>
@@ -2226,7 +2238,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:15" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:15" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="11">
         <v>23</v>
       </c>
@@ -2273,7 +2285,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:15" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:15" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
         <v>24</v>
       </c>
@@ -2320,7 +2332,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="8">
         <v>25</v>
       </c>
@@ -2367,7 +2379,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -2414,7 +2426,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -2461,7 +2473,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:15" s="13" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:15" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="13">
         <v>28</v>
       </c>
@@ -2508,7 +2520,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:15" s="13" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:15" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="13">
         <v>29</v>
       </c>
@@ -2555,7 +2567,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -2602,7 +2614,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -2649,7 +2661,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -2696,7 +2708,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -2743,7 +2755,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -2790,7 +2802,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -2837,7 +2849,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -2884,7 +2896,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:15" s="16" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:15" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="16">
         <v>37</v>
       </c>
@@ -2931,7 +2943,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -2978,7 +2990,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:15" s="16" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:15" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="16">
         <v>39</v>
       </c>
@@ -3025,7 +3037,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="16">
         <v>40</v>
       </c>
@@ -3072,7 +3084,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -3119,7 +3131,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="16">
         <v>42</v>
       </c>
@@ -3166,7 +3178,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>43</v>
       </c>
@@ -3213,7 +3225,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="19">
         <v>44</v>
       </c>
@@ -3260,7 +3272,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="19">
         <v>45</v>
       </c>
@@ -3307,7 +3319,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="19">
         <v>46</v>
       </c>
@@ -3354,7 +3366,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>47</v>
       </c>
@@ -3401,7 +3413,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="4">
         <v>48</v>
       </c>
@@ -3448,7 +3460,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
@@ -3495,7 +3507,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
@@ -3542,7 +3554,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>51</v>
       </c>
@@ -3589,7 +3601,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="36">
         <v>52</v>
       </c>
@@ -3636,7 +3648,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>53</v>
       </c>
@@ -3683,7 +3695,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="19">
         <v>54</v>
       </c>
@@ -3730,7 +3742,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>55</v>
       </c>
@@ -3777,7 +3789,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="19">
         <v>56</v>
       </c>
@@ -3824,7 +3836,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>57</v>
       </c>
@@ -3871,7 +3883,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="31">
         <v>58</v>
       </c>
@@ -3918,7 +3930,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="31">
         <v>59</v>
       </c>
@@ -3965,7 +3977,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="31">
         <v>60</v>
       </c>
@@ -4012,7 +4024,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="37">
         <v>61</v>
       </c>
@@ -4059,7 +4071,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="31">
         <v>62</v>
       </c>
@@ -4106,7 +4118,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="31">
         <v>63</v>
       </c>
@@ -4153,7 +4165,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="31">
         <v>64</v>
       </c>
@@ -4200,7 +4212,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="31">
         <v>65</v>
       </c>
@@ -4247,7 +4259,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="31">
         <v>66</v>
       </c>
@@ -4294,7 +4306,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="31">
         <v>67</v>
       </c>
@@ -4341,7 +4353,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="31">
         <v>68</v>
       </c>
@@ -4388,7 +4400,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="31">
         <v>69</v>
       </c>
@@ -4435,7 +4447,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="31">
         <v>70</v>
       </c>
@@ -4482,73 +4494,214 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A72">
+    <row r="72" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A72" s="31">
+        <v>71</v>
+      </c>
+      <c r="B72" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="C72" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="D72" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="E72" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="F72">
+        <v>27</v>
+      </c>
+      <c r="G72" s="21">
+        <v>5</v>
+      </c>
+      <c r="H72" s="21">
+        <v>4</v>
+      </c>
+      <c r="I72" s="19">
+        <v>1</v>
+      </c>
+      <c r="J72" s="19">
+        <v>1</v>
+      </c>
+      <c r="K72" s="19">
+        <v>2</v>
+      </c>
+      <c r="L72" s="21">
+        <v>13</v>
+      </c>
+      <c r="M72" s="19">
+        <v>2</v>
+      </c>
+      <c r="N72" s="19">
+        <v>1</v>
+      </c>
+      <c r="O72" s="19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A73" s="31">
+        <v>72</v>
+      </c>
+      <c r="B73" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="C73" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="D73" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="E73" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="F73">
+        <v>17</v>
+      </c>
+      <c r="G73" s="21">
+        <v>8</v>
+      </c>
+      <c r="H73" s="21">
+        <v>4</v>
+      </c>
+      <c r="I73" s="19">
+        <v>1</v>
+      </c>
+      <c r="J73" s="19">
+        <v>1</v>
+      </c>
+      <c r="K73" s="19">
+        <v>2</v>
+      </c>
+      <c r="L73" s="21">
+        <v>13</v>
+      </c>
+      <c r="M73" s="19">
+        <v>2</v>
+      </c>
+      <c r="N73" s="19">
+        <v>1</v>
+      </c>
+      <c r="O73" s="19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A74" s="31">
+        <v>73</v>
+      </c>
+      <c r="B74" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="C74" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="D74" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="E74" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="F74">
+        <v>17</v>
+      </c>
+      <c r="G74" s="21">
+        <v>9</v>
+      </c>
+      <c r="H74" s="21">
+        <v>4</v>
+      </c>
+      <c r="I74" s="19">
+        <v>1</v>
+      </c>
+      <c r="J74" s="19">
+        <v>1</v>
+      </c>
+      <c r="K74" s="19">
+        <v>2</v>
+      </c>
+      <c r="L74" s="21">
+        <v>13</v>
+      </c>
+      <c r="M74" s="19">
+        <v>2</v>
+      </c>
+      <c r="N74" s="19">
+        <v>1</v>
+      </c>
+      <c r="O74" s="19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A75">
         <v>10000</v>
       </c>
-      <c r="E72" t="s">
+      <c r="E75" t="s">
         <v>23</v>
       </c>
-      <c r="F72" t="s">
+      <c r="F75" t="s">
         <v>24</v>
       </c>
-      <c r="G72" t="s">
+      <c r="G75" t="s">
         <v>25</v>
       </c>
-      <c r="H72" t="s">
+      <c r="H75" t="s">
         <v>26</v>
       </c>
-      <c r="I72" t="s">
+      <c r="I75" t="s">
         <v>27</v>
       </c>
-      <c r="J72" t="s">
+      <c r="J75" t="s">
         <v>28</v>
       </c>
-      <c r="K72" t="s">
+      <c r="K75" t="s">
         <v>29</v>
       </c>
-      <c r="L72" t="s">
+      <c r="L75" t="s">
         <v>30</v>
       </c>
-      <c r="M72" t="s">
+      <c r="M75" t="s">
         <v>31</v>
       </c>
-      <c r="N72" t="s">
+      <c r="N75" t="s">
         <v>32</v>
       </c>
-      <c r="O72" t="s">
+      <c r="O75" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="F73">
-        <v>1</v>
-      </c>
-      <c r="G73">
-        <v>2</v>
-      </c>
-      <c r="H73">
+    <row r="76" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="F76">
+        <v>1</v>
+      </c>
+      <c r="G76">
+        <v>2</v>
+      </c>
+      <c r="H76">
         <v>3</v>
       </c>
-      <c r="I73">
+      <c r="I76">
         <v>4</v>
       </c>
-      <c r="J73">
+      <c r="J76">
         <v>5</v>
       </c>
-      <c r="K73">
+      <c r="K76">
         <v>6</v>
       </c>
-      <c r="L73">
+      <c r="L76">
         <v>7</v>
       </c>
-      <c r="M73">
+      <c r="M76">
         <v>8</v>
       </c>
-      <c r="N73">
+      <c r="N76">
         <v>9</v>
       </c>
-      <c r="O73">
+      <c r="O76">
         <v>10</v>
       </c>
     </row>
@@ -4561,9 +4714,9 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1025" width="8.7265625" customWidth="1"/>
+    <col min="1" max="1025" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
@@ -4574,12 +4727,12 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1025" width="8.7265625" customWidth="1"/>
+    <col min="1" max="1025" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>34</v>
       </c>
@@ -4587,7 +4740,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>33</v>
       </c>
@@ -4603,21 +4756,21 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:P27"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:P28"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.7265625" customWidth="1"/>
-    <col min="2" max="2" width="34.26953125" customWidth="1"/>
-    <col min="3" max="3" width="12.54296875" customWidth="1"/>
-    <col min="4" max="4" width="13.453125" customWidth="1"/>
-    <col min="5" max="5" width="7.54296875" customWidth="1"/>
-    <col min="6" max="7" width="7.7265625" customWidth="1"/>
-    <col min="8" max="8" width="13.1796875" customWidth="1"/>
-    <col min="9" max="9" width="12.54296875" customWidth="1"/>
-    <col min="10" max="1025" width="8.7265625" customWidth="1"/>
+    <col min="1" max="1" width="8.7109375" customWidth="1"/>
+    <col min="2" max="2" width="34.28515625" customWidth="1"/>
+    <col min="3" max="3" width="12.5703125" customWidth="1"/>
+    <col min="4" max="4" width="13.42578125" customWidth="1"/>
+    <col min="5" max="5" width="7.5703125" customWidth="1"/>
+    <col min="6" max="7" width="7.7109375" customWidth="1"/>
+    <col min="8" max="8" width="13.140625" customWidth="1"/>
+    <col min="9" max="9" width="12.5703125" customWidth="1"/>
+    <col min="10" max="1025" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>34</v>
       </c>
@@ -4667,7 +4820,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -4717,7 +4870,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>51</v>
       </c>
@@ -4767,7 +4920,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>53</v>
       </c>
@@ -4818,7 +4971,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>55</v>
       </c>
@@ -4868,7 +5021,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>57</v>
       </c>
@@ -4918,7 +5071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>58</v>
       </c>
@@ -4968,7 +5121,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>59</v>
       </c>
@@ -5018,7 +5171,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>61</v>
       </c>
@@ -5068,7 +5221,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>63</v>
       </c>
@@ -5118,7 +5271,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>65</v>
       </c>
@@ -5168,7 +5321,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>67</v>
       </c>
@@ -5219,7 +5372,7 @@
         <v>5.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>69</v>
       </c>
@@ -5269,7 +5422,7 @@
         <v>5.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>71</v>
       </c>
@@ -5320,7 +5473,7 @@
         <v>2.5000000000000001E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>73</v>
       </c>
@@ -5371,7 +5524,7 @@
         <v>3.7499999999999999E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>148</v>
       </c>
@@ -5422,7 +5575,7 @@
         <v>3.7499999999999999E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>150</v>
       </c>
@@ -5472,7 +5625,7 @@
         <v>3.7499999999999999E-3</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>152</v>
       </c>
@@ -5523,7 +5676,7 @@
         <v>3.7499999999999999E-3</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>154</v>
       </c>
@@ -5573,7 +5726,7 @@
         <v>3.8E-3</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>157</v>
       </c>
@@ -5620,11 +5773,11 @@
         <v>0.08</v>
       </c>
       <c r="P20">
-        <f t="shared" ref="P20:P26" si="0">1.5/400</f>
+        <f t="shared" ref="P20:P28" si="0">1.5/400</f>
         <v>3.7499999999999999E-3</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>159</v>
       </c>
@@ -5675,7 +5828,7 @@
         <v>3.7499999999999999E-3</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>161</v>
       </c>
@@ -5726,7 +5879,7 @@
         <v>3.7499999999999999E-3</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>162</v>
       </c>
@@ -5777,7 +5930,7 @@
         <v>3.7499999999999999E-3</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>164</v>
       </c>
@@ -5828,7 +5981,7 @@
         <v>3.7499999999999999E-3</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>165</v>
       </c>
@@ -5879,7 +6032,7 @@
         <v>3.7499999999999999E-3</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>168</v>
       </c>
@@ -5930,7 +6083,7 @@
         <v>3.7499999999999999E-3</v>
       </c>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>170</v>
       </c>
@@ -5978,6 +6131,57 @@
       </c>
       <c r="P27">
         <f>1.5/400</f>
+        <v>3.7499999999999999E-3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>171</v>
+      </c>
+      <c r="B28" t="s">
+        <v>172</v>
+      </c>
+      <c r="C28">
+        <v>1</v>
+      </c>
+      <c r="D28" s="28">
+        <v>0.4</v>
+      </c>
+      <c r="E28">
+        <v>0</v>
+      </c>
+      <c r="F28">
+        <v>0</v>
+      </c>
+      <c r="G28">
+        <v>1.7299999999999999E-2</v>
+      </c>
+      <c r="H28">
+        <v>1</v>
+      </c>
+      <c r="I28" s="28">
+        <v>0.4</v>
+      </c>
+      <c r="J28">
+        <v>0</v>
+      </c>
+      <c r="K28">
+        <v>0</v>
+      </c>
+      <c r="L28">
+        <v>1.7299999999999999E-2</v>
+      </c>
+      <c r="M28">
+        <v>0.995</v>
+      </c>
+      <c r="N28">
+        <v>0.995</v>
+      </c>
+      <c r="O28">
+        <v>0.08</v>
+      </c>
+      <c r="P28">
+        <f t="shared" si="0"/>
         <v>3.7499999999999999E-3</v>
       </c>
     </row>
@@ -5989,13 +6193,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F8"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1025" width="8.7265625" customWidth="1"/>
+    <col min="1" max="1025" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>34</v>
       </c>
@@ -6012,7 +6216,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>79</v>
       </c>
@@ -6030,7 +6234,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>81</v>
       </c>
@@ -6050,7 +6254,7 @@
         <v>0.66666666666666674</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>82</v>
       </c>
@@ -6069,7 +6273,7 @@
         <v>1.4</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>83</v>
       </c>
@@ -6088,7 +6292,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>84</v>
       </c>
@@ -6107,7 +6311,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>85</v>
       </c>
@@ -6128,7 +6332,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>86</v>
       </c>
@@ -6148,6 +6352,44 @@
       </c>
       <c r="F8">
         <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>173</v>
+      </c>
+      <c r="B9" t="s">
+        <v>80</v>
+      </c>
+      <c r="C9">
+        <f>E9/400</f>
+        <v>1.5E-3</v>
+      </c>
+      <c r="D9">
+        <f>E9/400</f>
+        <v>1.5E-3</v>
+      </c>
+      <c r="E9">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>174</v>
+      </c>
+      <c r="B10" t="s">
+        <v>80</v>
+      </c>
+      <c r="C10">
+        <f>E10/400</f>
+        <v>6.0000000000000001E-3</v>
+      </c>
+      <c r="D10">
+        <f>E10/400</f>
+        <v>6.0000000000000001E-3</v>
+      </c>
+      <c r="E10">
+        <v>2.4</v>
       </c>
     </row>
   </sheetData>
@@ -6159,16 +6401,16 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.7265625" customWidth="1"/>
-    <col min="2" max="2" width="14.1796875" customWidth="1"/>
-    <col min="3" max="3" width="17.7265625" customWidth="1"/>
-    <col min="4" max="4" width="13.54296875" customWidth="1"/>
-    <col min="5" max="1025" width="8.7265625" customWidth="1"/>
+    <col min="1" max="1" width="8.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.140625" customWidth="1"/>
+    <col min="3" max="3" width="17.7109375" customWidth="1"/>
+    <col min="4" max="4" width="13.5703125" customWidth="1"/>
+    <col min="5" max="1025" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>34</v>
       </c>
@@ -6191,7 +6433,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>26</v>
       </c>
@@ -6211,7 +6453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>94</v>
       </c>
@@ -6231,7 +6473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>95</v>
       </c>
@@ -6251,7 +6493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>96</v>
       </c>
@@ -6271,7 +6513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>97</v>
       </c>
@@ -6291,7 +6533,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>98</v>
       </c>
@@ -6320,12 +6562,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1025" width="8.7265625" customWidth="1"/>
+    <col min="1" max="1025" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>34</v>
       </c>
@@ -6339,7 +6581,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>102</v>
       </c>
@@ -6362,17 +6604,17 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="C1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1025" width="8.7265625" customWidth="1"/>
+    <col min="1" max="1025" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C1" s="25" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="2" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C2">
         <v>2.5000000000000001E-3</v>
       </c>
@@ -6386,15 +6628,15 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.7265625" customWidth="1"/>
-    <col min="2" max="4" width="15.1796875" customWidth="1"/>
-    <col min="5" max="5" width="17.7265625" customWidth="1"/>
-    <col min="6" max="1025" width="8.7265625" customWidth="1"/>
+    <col min="1" max="1" width="8.7109375" customWidth="1"/>
+    <col min="2" max="4" width="15.140625" customWidth="1"/>
+    <col min="5" max="5" width="17.7109375" customWidth="1"/>
+    <col min="6" max="1025" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>34</v>
       </c>
@@ -6411,7 +6653,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>29</v>
       </c>
@@ -6428,7 +6670,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>109</v>
       </c>
@@ -6454,16 +6696,16 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:R18"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="7" width="8.7265625" customWidth="1"/>
-    <col min="8" max="8" width="11.453125"/>
-    <col min="9" max="13" width="8.7265625" customWidth="1"/>
+    <col min="1" max="7" width="8.7109375" customWidth="1"/>
+    <col min="8" max="8" width="11.42578125"/>
+    <col min="9" max="13" width="8.7109375" customWidth="1"/>
     <col min="14" max="14" width="11" customWidth="1"/>
-    <col min="15" max="1025" width="8.7265625" customWidth="1"/>
+    <col min="15" max="1025" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>34</v>
       </c>
@@ -6519,7 +6761,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>30</v>
       </c>
@@ -6563,7 +6805,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>129</v>
       </c>
@@ -6607,7 +6849,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>131</v>
       </c>
@@ -6651,7 +6893,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>132</v>
       </c>
@@ -6695,7 +6937,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>134</v>
       </c>
@@ -6739,7 +6981,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>135</v>
       </c>
@@ -6783,7 +7025,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>136</v>
       </c>
@@ -6827,7 +7069,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>137</v>
       </c>
@@ -6871,7 +7113,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>138</v>
       </c>
@@ -6915,7 +7157,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>139</v>
       </c>
@@ -6959,7 +7201,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>140</v>
       </c>
@@ -7003,7 +7245,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>141</v>
       </c>
@@ -7047,7 +7289,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>142</v>
       </c>
@@ -7091,7 +7333,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>143</v>
       </c>
@@ -7135,7 +7377,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>144</v>
       </c>
@@ -7179,7 +7421,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>156</v>
       </c>
@@ -7223,7 +7465,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="C18" s="1"/>
     </row>
   </sheetData>
@@ -7235,12 +7477,12 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1025" width="8.7265625" customWidth="1"/>
+    <col min="1" max="1025" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>34</v>
       </c>
@@ -7248,7 +7490,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>31</v>
       </c>
@@ -7256,7 +7498,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>146</v>
       </c>

</xml_diff>